<commit_message>
thêm mã phòng ban vào câu hỏi import
</commit_message>
<xml_diff>
--- a/client/public/templates/Mau_Import_Cau_Hoi_Z176.xlsx
+++ b/client/public/templates/Mau_Import_Cau_Hoi_Z176.xlsx
@@ -475,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F20"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -492,6 +492,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -499,6 +500,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
@@ -610,7 +612,7 @@
     <row r="9" ht="44" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Bộ phận</t>
+          <t>Mã bộ phận</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
@@ -620,7 +622,7 @@
       </c>
       <c r="C9" s="4" t="inlineStr">
         <is>
-          <t>Đúng tên 1 trong 9 phòng ban hiện có trong hệ thống</t>
+          <t>Mã của 1 bộ phận ĐÃ CÓ trong hệ thống, vd: HCHC, CNTT, KTCK</t>
         </is>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -630,14 +632,14 @@
       </c>
       <c r="E9" s="4" t="inlineStr">
         <is>
-          <t>BẮT BUỘC nếu Phạm vi = riêng. Bỏ trống nếu Phạm vi = chung.</t>
+          <t>BẮT BUỘC nếu Phạm vi = riêng. Hệ thống tìm bộ phận theo MÃ này (không phân biệt hoa/thường). Bỏ trống nếu Phạm vi = chung.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="44" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>Loại</t>
+          <t>Bộ phận</t>
         </is>
       </c>
       <c r="B10" s="4" t="inlineStr">
@@ -647,20 +649,24 @@
       </c>
       <c r="C10" s="4" t="inlineStr">
         <is>
-          <t>lý thuyết  hoặc  bài tập</t>
+          <t>Tên bộ phận (cho người đọc dễ hiểu)</t>
         </is>
       </c>
       <c r="D10" s="4" t="inlineStr">
         <is>
-          <t>lý thuyết</t>
-        </is>
-      </c>
-      <c r="E10" s="4" t="inlineStr"/>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E10" s="4" t="inlineStr">
+        <is>
+          <t>Hệ thống KHÔNG dùng tên để tìm bộ phận. Chỉ khi Mã bộ phận chưa tồn tại: tên + mã được dùng để tạo bộ phận mới ở bước xem trước (nếu bạn tick tạo).</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="44" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Đáp án</t>
+          <t>Loại</t>
         </is>
       </c>
       <c r="B11" s="4" t="inlineStr">
@@ -670,24 +676,20 @@
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>chọn 1  hoặc  chọn nhiều</t>
+          <t>lý thuyết  hoặc  bài tập</t>
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr">
         <is>
-          <t>chọn 1</t>
-        </is>
-      </c>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>Phải khớp với số lượng đáp án đúng khai ở cột "Đáp án đúng" — nếu chọn 1 thì chỉ được ghi đúng 1 số ở cột đó.</t>
-        </is>
-      </c>
+          <t>lý thuyết</t>
+        </is>
+      </c>
+      <c r="E11" s="4" t="inlineStr"/>
     </row>
     <row r="12" ht="44" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>Độ khó</t>
+          <t>Đáp án</t>
         </is>
       </c>
       <c r="B12" s="4" t="inlineStr">
@@ -697,112 +699,148 @@
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>dễ, trung bình, khó</t>
+          <t>chọn 1  hoặc  chọn nhiều</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
         <is>
-          <t>trung bình</t>
-        </is>
-      </c>
-      <c r="E12" s="4" t="inlineStr"/>
+          <t>chọn 1</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Phải khớp với số lượng đáp án đúng khai ở cột "Đáp án đúng" — nếu chọn 1 thì chỉ được ghi đúng 1 số ở cột đó.</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="44" customHeight="1">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>Lựa chọn 1 … Lựa chọn 8</t>
+          <t>Độ khó</t>
         </is>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Có (ít nhất 2)</t>
+          <t>Không</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Nội dung từng phương án trả lời</t>
+          <t>dễ, trung bình, khó</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="E13" s="4" t="inlineStr">
-        <is>
-          <t>Cần điền tối thiểu Lựa chọn 1 và Lựa chọn 2. Có thể dùng tới Lựa chọn 8 nếu câu hỏi nhiều phương án.</t>
-        </is>
-      </c>
+          <t>trung bình</t>
+        </is>
+      </c>
+      <c r="E13" s="4" t="inlineStr"/>
     </row>
     <row r="14" ht="44" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
+          <t>Lựa chọn 1 … Lựa chọn 8</t>
+        </is>
+      </c>
+      <c r="B14" s="4" t="inlineStr">
+        <is>
+          <t>Có (ít nhất 2)</t>
+        </is>
+      </c>
+      <c r="C14" s="4" t="inlineStr">
+        <is>
+          <t>Nội dung từng phương án trả lời</t>
+        </is>
+      </c>
+      <c r="D14" s="4" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="E14" s="4" t="inlineStr">
+        <is>
+          <t>Cần điền tối thiểu Lựa chọn 1 và Lựa chọn 2. Có thể dùng tới Lựa chọn 8 nếu câu hỏi nhiều phương án.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="44" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
+        <is>
           <t>Đáp án đúng</t>
         </is>
       </c>
-      <c r="B14" s="4" t="inlineStr">
+      <c r="B15" s="4" t="inlineStr">
         <is>
           <t>Có</t>
         </is>
       </c>
-      <c r="C14" s="4" t="inlineStr">
+      <c r="C15" s="4" t="inlineStr">
         <is>
           <t>Số thứ tự phương án đúng, vd: 1  hoặc  1,3 (nếu chọn nhiều)</t>
         </is>
       </c>
-      <c r="D14" s="4" t="inlineStr">
+      <c r="D15" s="4" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E14" s="4" t="inlineStr">
+      <c r="E15" s="4" t="inlineStr">
         <is>
           <t>Số tương ứng với Lựa chọn N (Lựa chọn 1 → số 1, Lựa chọn 2 → số 2...). Nếu Đáp án = chọn 1 thì chỉ được ghi đúng 1 số.</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+    <row r="16"/>
+    <row r="17">
+      <c r="A17" s="5" t="inlineStr">
         <is>
           <t>Lưu ý quan trọng:</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>• Dòng đầu tiên (header) không được đổi tên cột — gõ đúng chính xác tên cột tiếng Việt như trong file này (có dấu đầy đủ).</t>
         </is>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>• Mỗi dòng trong sheet "Câu hỏi" = 1 câu hỏi. Xem 2 dòng ví dụ có sẵn để tham khảo định dạng.</t>
+          <t>• Dòng đầu tiên (header) không được đổi tên cột — gõ đúng chính xác tên cột tiếng Việt như trong file này (có dấu đầy đủ).</t>
         </is>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>• Nếu 1 dòng bị lỗi (vd thiếu đáp án đúng, sai tên phòng ban...), hệ thống sẽ bỏ qua đúng dòng đó và báo lỗi chi tiết theo số dòng — các dòng còn lại vẫn được import bình thường.</t>
+          <t>• Mỗi dòng trong sheet "Câu hỏi" = 1 câu hỏi. Sheet có 7 dòng ví dụ: câu Chung, câu Riêng (có đủ Mã + Tên, chỉ có Mã), câu chọn 1 / chọn nhiều, và 1 câu dùng cho 2 bộ phận (viết lặp lại). XÓA các dòng ví dụ trước khi nhập dữ liệu thật.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>• Kiểm tra tên phòng ban và tên chủ đề trùng khớp với dữ liệu đã có trong hệ thống trước khi import số lượng lớn, tránh tạo trùng chủ đề do lỗi chính tả.</t>
+          <t>• Nếu 1 dòng bị lỗi (vd thiếu đáp án đúng, sai mã bộ phận...), hệ thống sẽ bỏ qua đúng dòng đó và báo lỗi chi tiết theo số dòng — các dòng còn lại vẫn được import bình thường.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>• Câu dùng cho nhiều bộ phận: viết lặp lại, mỗi bộ phận 1 dòng (mỗi dòng 1 Mã bộ phận). Câu dùng cho mọi bộ phận thì để Phạm vi = chung.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>• Kiểm tra Mã bộ phận và tên chủ đề trùng khớp với dữ liệu đã có trong hệ thống trước khi import số lượng lớn, tránh tạo trùng do lỗi chính tả.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="7">
     <mergeCell ref="A19:F19"/>
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A17:F17"/>
+    <mergeCell ref="A22:F22"/>
     <mergeCell ref="A18:F18"/>
     <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A21:F21"/>
     <mergeCell ref="A20:F20"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -815,25 +853,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:Q8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="20" customWidth="1" min="9" max="9"/>
     <col width="20" customWidth="1" min="10" max="10"/>
     <col width="20" customWidth="1" min="11" max="11"/>
-    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
     <col width="16" customWidth="1" min="13" max="13"/>
     <col width="16" customWidth="1" min="14" max="14"/>
     <col width="16" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -854,65 +893,70 @@
       </c>
       <c r="D1" s="7" t="inlineStr">
         <is>
+          <t>Mã bộ phận</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
           <t>Bộ phận</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="F1" s="7" t="inlineStr">
         <is>
           <t>Loại</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="G1" s="7" t="inlineStr">
         <is>
           <t>Đáp án</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="H1" s="7" t="inlineStr">
         <is>
           <t>Độ khó</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="I1" s="7" t="inlineStr">
         <is>
           <t>Lựa chọn 1</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
+      <c r="J1" s="7" t="inlineStr">
         <is>
           <t>Lựa chọn 2</t>
         </is>
       </c>
-      <c r="J1" s="7" t="inlineStr">
+      <c r="K1" s="7" t="inlineStr">
         <is>
           <t>Lựa chọn 3</t>
         </is>
       </c>
-      <c r="K1" s="7" t="inlineStr">
+      <c r="L1" s="7" t="inlineStr">
         <is>
           <t>Lựa chọn 4</t>
         </is>
       </c>
-      <c r="L1" s="7" t="inlineStr">
+      <c r="M1" s="7" t="inlineStr">
         <is>
           <t>Lựa chọn 5</t>
         </is>
       </c>
-      <c r="M1" s="7" t="inlineStr">
+      <c r="N1" s="7" t="inlineStr">
         <is>
           <t>Lựa chọn 6</t>
         </is>
       </c>
-      <c r="N1" s="7" t="inlineStr">
+      <c r="O1" s="7" t="inlineStr">
         <is>
           <t>Lựa chọn 7</t>
         </is>
       </c>
-      <c r="O1" s="7" t="inlineStr">
+      <c r="P1" s="7" t="inlineStr">
         <is>
           <t>Lựa chọn 8</t>
         </is>
       </c>
-      <c r="P1" s="7" t="inlineStr">
+      <c r="Q1" s="7" t="inlineStr">
         <is>
           <t>Đáp án đúng</t>
         </is>
@@ -921,12 +965,12 @@
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
         <is>
-          <t>Điều lệnh đội ngũ</t>
+          <t>An toàn lao động</t>
         </is>
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>Khẩu lệnh "Nghiêm!" được dùng trong trường hợp nào?</t>
+          <t>Khi phát hiện đám cháy nhỏ tại nơi làm việc, việc đầu tiên cần làm là gì?</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
@@ -934,47 +978,48 @@
           <t>chung</t>
         </is>
       </c>
-      <c r="D2" s="4" t="inlineStr"/>
-      <c r="E2" s="4" t="inlineStr">
+      <c r="D2" s="4" t="n"/>
+      <c r="E2" s="4" t="n"/>
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>lý thuyết</t>
         </is>
       </c>
-      <c r="F2" s="4" t="inlineStr">
+      <c r="G2" s="4" t="inlineStr">
         <is>
           <t>chọn 1</t>
         </is>
       </c>
-      <c r="G2" s="4" t="inlineStr">
+      <c r="H2" s="4" t="inlineStr">
         <is>
           <t>dễ</t>
         </is>
       </c>
-      <c r="H2" s="4" t="inlineStr">
-        <is>
-          <t>Khi bắt đầu buổi tập hợp đội ngũ</t>
-        </is>
-      </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Khi giải tán đội hình</t>
+          <t>Báo động và thông báo cho mọi người xung quanh</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">
         <is>
-          <t>Khi nghỉ giải lao</t>
+          <t>Tiếp tục làm việc như bình thường</t>
         </is>
       </c>
       <c r="K2" s="4" t="inlineStr">
         <is>
-          <t>Khi báo cáo cấp trên</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr"/>
-      <c r="M2" s="4" t="inlineStr"/>
-      <c r="N2" s="4" t="inlineStr"/>
-      <c r="O2" s="4" t="inlineStr"/>
-      <c r="P2" s="4" t="inlineStr">
+          <t>Chụp ảnh đăng lên mạng xã hội</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>Rời đi mà không báo cho ai</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="n"/>
+      <c r="N2" s="4" t="n"/>
+      <c r="O2" s="4" t="n"/>
+      <c r="P2" s="4" t="n"/>
+      <c r="Q2" s="4" t="inlineStr">
         <is>
           <t>1</t>
         </is>
@@ -983,66 +1028,414 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
+          <t>An toàn lao động</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Những việc nào sau đây giúp phòng ngừa tai nạn lao động?</t>
+        </is>
+      </c>
+      <c r="C3" s="4" t="inlineStr">
+        <is>
+          <t>chung</t>
+        </is>
+      </c>
+      <c r="D3" s="4" t="n"/>
+      <c r="E3" s="4" t="n"/>
+      <c r="F3" s="4" t="inlineStr">
+        <is>
+          <t>bài tập</t>
+        </is>
+      </c>
+      <c r="G3" s="4" t="inlineStr">
+        <is>
+          <t>chọn nhiều</t>
+        </is>
+      </c>
+      <c r="H3" s="4" t="inlineStr">
+        <is>
+          <t>trung bình</t>
+        </is>
+      </c>
+      <c r="I3" s="4" t="inlineStr">
+        <is>
+          <t>Đội mũ bảo hộ khi vào xưởng</t>
+        </is>
+      </c>
+      <c r="J3" s="4" t="inlineStr">
+        <is>
+          <t>Tháo thiết bị bảo vệ để làm nhanh hơn</t>
+        </is>
+      </c>
+      <c r="K3" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra máy trước khi vận hành</t>
+        </is>
+      </c>
+      <c r="L3" s="4" t="inlineStr">
+        <is>
+          <t>Làm việc khi đang rất mệt mỏi</t>
+        </is>
+      </c>
+      <c r="M3" s="4" t="n"/>
+      <c r="N3" s="4" t="n"/>
+      <c r="O3" s="4" t="n"/>
+      <c r="P3" s="4" t="n"/>
+      <c r="Q3" s="4" t="inlineStr">
+        <is>
+          <t>1,3</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Công nghệ thông tin</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Mật khẩu nào sau đây an toàn nhất?</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>riêng</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>CNTT</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Công nghệ thông tin</t>
+        </is>
+      </c>
+      <c r="F4" s="4" t="inlineStr">
+        <is>
+          <t>lý thuyết</t>
+        </is>
+      </c>
+      <c r="G4" s="4" t="inlineStr">
+        <is>
+          <t>chọn 1</t>
+        </is>
+      </c>
+      <c r="H4" s="4" t="inlineStr">
+        <is>
+          <t>dễ</t>
+        </is>
+      </c>
+      <c r="I4" s="4" t="inlineStr">
+        <is>
+          <t>12345678</t>
+        </is>
+      </c>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>Ngày sinh của bản thân</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>Chuỗi dài gồm chữ hoa, chữ thường, số và ký tự đặc biệt</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>Tên đăng nhập của tài khoản</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="n"/>
+      <c r="N4" s="4" t="n"/>
+      <c r="O4" s="4" t="n"/>
+      <c r="P4" s="4" t="n"/>
+      <c r="Q4" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Công nghệ thông tin</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Hành động nào giúp giảm nguy cơ bị lừa đảo qua email?</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>riêng</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>CNTT</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="n"/>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>lý thuyết</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>chọn nhiều</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>khó</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra kỹ địa chỉ người gửi</t>
+        </is>
+      </c>
+      <c r="J5" s="4" t="inlineStr">
+        <is>
+          <t>Mở mọi tệp đính kèm cho nhanh</t>
+        </is>
+      </c>
+      <c r="K5" s="4" t="inlineStr">
+        <is>
+          <t>Không nhập mật khẩu qua đường dẫn lạ</t>
+        </is>
+      </c>
+      <c r="L5" s="4" t="inlineStr">
+        <is>
+          <t>Chuyển tiếp email cho tất cả đồng nghiệp</t>
+        </is>
+      </c>
+      <c r="M5" s="4" t="n"/>
+      <c r="N5" s="4" t="n"/>
+      <c r="O5" s="4" t="n"/>
+      <c r="P5" s="4" t="n"/>
+      <c r="Q5" s="4" t="inlineStr">
+        <is>
+          <t>1,3</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Nghiệp vụ hành chính</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="inlineStr">
+        <is>
+          <t>Khi tiếp nhận nhân viên mới, hồ sơ nào cần hoàn thiện đầu tiên?</t>
+        </is>
+      </c>
+      <c r="C6" s="4" t="inlineStr">
+        <is>
+          <t>riêng</t>
+        </is>
+      </c>
+      <c r="D6" s="4" t="inlineStr">
+        <is>
+          <t>HCNS</t>
+        </is>
+      </c>
+      <c r="E6" s="4" t="inlineStr">
+        <is>
+          <t>Hành chính - Nhân sự</t>
+        </is>
+      </c>
+      <c r="F6" s="4" t="inlineStr">
+        <is>
+          <t>lý thuyết</t>
+        </is>
+      </c>
+      <c r="G6" s="4" t="inlineStr">
+        <is>
+          <t>chọn 1</t>
+        </is>
+      </c>
+      <c r="H6" s="4" t="inlineStr">
+        <is>
+          <t>trung bình</t>
+        </is>
+      </c>
+      <c r="I6" s="4" t="inlineStr">
+        <is>
+          <t>Hồ sơ cá nhân và thông tin liên hệ</t>
+        </is>
+      </c>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>Bảng giá vật tư</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>Lịch bảo trì máy</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>Báo cáo tài chính năm</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="n"/>
+      <c r="N6" s="4" t="n"/>
+      <c r="O6" s="4" t="n"/>
+      <c r="P6" s="4" t="n"/>
+      <c r="Q6" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>An toàn lao động</t>
+        </is>
+      </c>
+      <c r="B7" s="4" t="inlineStr">
+        <is>
+          <t>Trước khi vận hành thiết bị nâng hạ, người vận hành phải làm gì trước tiên?</t>
+        </is>
+      </c>
+      <c r="C7" s="4" t="inlineStr">
+        <is>
+          <t>riêng</t>
+        </is>
+      </c>
+      <c r="D7" s="4" t="inlineStr">
+        <is>
+          <t>KTCK</t>
+        </is>
+      </c>
+      <c r="E7" s="4" t="inlineStr">
+        <is>
           <t>Kỹ thuật cơ khí</t>
         </is>
       </c>
-      <c r="B3" s="4" t="inlineStr">
-        <is>
-          <t>Những dụng cụ nào sau đây dùng để đo kích thước chi tiết cơ khí? (chọn nhiều)</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
+      <c r="F7" s="4" t="inlineStr">
+        <is>
+          <t>bài tập</t>
+        </is>
+      </c>
+      <c r="G7" s="4" t="inlineStr">
+        <is>
+          <t>chọn 1</t>
+        </is>
+      </c>
+      <c r="H7" s="4" t="inlineStr">
+        <is>
+          <t>trung bình</t>
+        </is>
+      </c>
+      <c r="I7" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra tình trạng thiết bị và khu vực xung quanh</t>
+        </is>
+      </c>
+      <c r="J7" s="4" t="inlineStr">
+        <is>
+          <t>Vận hành ngay để kịp tiến độ</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>Nhờ người chưa được huấn luyện vận hành thay</t>
+        </is>
+      </c>
+      <c r="L7" s="4" t="inlineStr">
+        <is>
+          <t>Bỏ qua việc kiểm tra vì máy mới</t>
+        </is>
+      </c>
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4" t="n"/>
+      <c r="O7" s="4" t="n"/>
+      <c r="P7" s="4" t="n"/>
+      <c r="Q7" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="4" t="inlineStr">
+        <is>
+          <t>An toàn lao động</t>
+        </is>
+      </c>
+      <c r="B8" s="4" t="inlineStr">
+        <is>
+          <t>Trước khi vận hành thiết bị nâng hạ, người vận hành phải làm gì trước tiên?</t>
+        </is>
+      </c>
+      <c r="C8" s="4" t="inlineStr">
         <is>
           <t>riêng</t>
         </is>
       </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Phòng Kỹ thuật</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
+      <c r="D8" s="4" t="inlineStr">
+        <is>
+          <t>HCHC</t>
+        </is>
+      </c>
+      <c r="E8" s="4" t="inlineStr">
+        <is>
+          <t>Hành chính hậu cần</t>
+        </is>
+      </c>
+      <c r="F8" s="4" t="inlineStr">
         <is>
           <t>bài tập</t>
         </is>
       </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>chọn nhiều</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G8" s="4" t="inlineStr">
+        <is>
+          <t>chọn 1</t>
+        </is>
+      </c>
+      <c r="H8" s="4" t="inlineStr">
         <is>
           <t>trung bình</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Thước cặp</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Panme</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Búa</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Đồng hồ so</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr"/>
-      <c r="M3" s="4" t="inlineStr"/>
-      <c r="N3" s="4" t="inlineStr"/>
-      <c r="O3" s="4" t="inlineStr"/>
-      <c r="P3" s="4" t="inlineStr">
-        <is>
-          <t>1,2,4</t>
+      <c r="I8" s="4" t="inlineStr">
+        <is>
+          <t>Kiểm tra tình trạng thiết bị và khu vực xung quanh</t>
+        </is>
+      </c>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>Vận hành ngay để kịp tiến độ</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>Nhờ người chưa được huấn luyện vận hành thay</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>Bỏ qua việc kiểm tra vì máy mới</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="n"/>
+      <c r="N8" s="4" t="n"/>
+      <c r="O8" s="4" t="n"/>
+      <c r="P8" s="4" t="n"/>
+      <c r="Q8" s="4" t="inlineStr">
+        <is>
+          <t>1</t>
         </is>
       </c>
     </row>
@@ -1051,13 +1444,13 @@
     <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"chung,riêng"</formula1>
     </dataValidation>
-    <dataValidation sqref="E2:E200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"lý thuyết,bài tập"</formula1>
     </dataValidation>
-    <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="G2:G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"chọn 1,chọn nhiều"</formula1>
     </dataValidation>
-    <dataValidation sqref="G2:G200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="H2:H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"dễ,trung bình,khó"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>